<commit_message>
Finished bluetooth testing and placed results into technical report.
</commit_message>
<xml_diff>
--- a/testing/battery_test.xlsx
+++ b/testing/battery_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arshsingh/Desktop/Spring_2025/BME_554/ecg-temp-ble-project/testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA7FE59E-82DD-624B-9897-27236B723438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E06330-B5CB-EB4B-A5AF-A7C2D8095A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{157B1088-A0BA-9E45-9B40-F1125BBB911F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="8">
   <si>
     <t>High</t>
   </si>
@@ -54,6 +54,12 @@
   </si>
   <si>
     <t>Trial 3</t>
+  </si>
+  <si>
+    <t>Trial 4</t>
+  </si>
+  <si>
+    <t>Trial 5</t>
   </si>
 </sst>
 </file>
@@ -425,18 +431,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FAD543C-B4F2-5044-99A9-2BE8FACFAAE2}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -450,16 +456,28 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>0</v>
       </c>
@@ -473,16 +491,28 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G3">
         <v>1000</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3">
+        <v>1000</v>
+      </c>
+      <c r="I3">
+        <v>1000</v>
+      </c>
+      <c r="J3">
+        <v>1000</v>
+      </c>
+      <c r="K3">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>0.5</v>
       </c>
@@ -496,16 +526,28 @@
         <v>170</v>
       </c>
       <c r="E4">
+        <v>180</v>
+      </c>
+      <c r="F4">
+        <v>170</v>
+      </c>
+      <c r="G4">
         <v>830</v>
       </c>
-      <c r="F4">
+      <c r="H4">
         <v>820</v>
       </c>
-      <c r="G4">
+      <c r="I4">
         <v>820</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="J4">
+        <v>830</v>
+      </c>
+      <c r="K4">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -519,16 +561,28 @@
         <v>330</v>
       </c>
       <c r="E5">
+        <v>330</v>
+      </c>
+      <c r="F5">
+        <v>330</v>
+      </c>
+      <c r="G5">
         <v>660</v>
       </c>
-      <c r="F5">
+      <c r="H5">
         <v>660</v>
       </c>
-      <c r="G5">
+      <c r="I5">
         <v>670</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="J5">
+        <v>670</v>
+      </c>
+      <c r="K5">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1.5</v>
       </c>
@@ -550,8 +604,20 @@
       <c r="G6">
         <v>500</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6">
+        <v>500</v>
+      </c>
+      <c r="I6">
+        <v>500</v>
+      </c>
+      <c r="J6">
+        <v>500</v>
+      </c>
+      <c r="K6">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2</v>
       </c>
@@ -565,16 +631,28 @@
         <v>660</v>
       </c>
       <c r="E7">
-        <v>340</v>
+        <v>640</v>
       </c>
       <c r="F7">
-        <v>360</v>
+        <v>660</v>
       </c>
       <c r="G7">
         <v>340</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7">
+        <v>360</v>
+      </c>
+      <c r="I7">
+        <v>340</v>
+      </c>
+      <c r="J7">
+        <v>340</v>
+      </c>
+      <c r="K7">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2.5</v>
       </c>
@@ -588,16 +666,28 @@
         <v>830</v>
       </c>
       <c r="E8">
-        <v>170</v>
+        <v>840</v>
       </c>
       <c r="F8">
-        <v>160</v>
+        <v>830</v>
       </c>
       <c r="G8">
         <v>170</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8">
+        <v>160</v>
+      </c>
+      <c r="I8">
+        <v>170</v>
+      </c>
+      <c r="J8">
+        <v>160</v>
+      </c>
+      <c r="K8">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>3</v>
       </c>
@@ -611,12 +701,24 @@
         <v>1000</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
         <v>0</v>
       </c>
     </row>

</xml_diff>